<commit_message>
fix: sample import spreadsheet no longer repeats a seeded sample dish (#344)
PE-11: "Fresh Lime Soda" (also in every new tenant's sample menu) renamed
"Sweet Lime Soda", so the template imports cleanly on a fresh tenant.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/menu-import-template.xlsx
+++ b/public/menu-import-template.xlsx
@@ -932,12 +932,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Fresh Lime Soda</t>
+          <t>Sweet Lime Soda</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Lime Soda</t>
+          <t>Sweet Lime</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">

</xml_diff>